<commit_message>
fix: bypass isDeleted mongoose hook when importing excel to allow updating/restoring soft-deleted products
</commit_message>
<xml_diff>
--- a/backend/uploads/Sample_Products.xlsx
+++ b/backend/uploads/Sample_Products.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tranm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NNPTUD_DoAn\backend\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{5EE9C431-EC15-43C7-921A-E3750169D068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -1218,7 +1218,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1226,7 +1226,7 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1596,12 +1596,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N101"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="130.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="130.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>65</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>69</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>72</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>77</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>80</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>83</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>88</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>94</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>102</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>106</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>109</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>113</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>116</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>119</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>121</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>124</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>127</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>129</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>132</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>134</v>
       </c>
@@ -2921,7 +2921,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>136</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>139</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>141</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>144</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>147</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>150</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>152</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>154</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>156</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>159</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>162</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>164</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>167</v>
       </c>
@@ -3493,7 +3493,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>169</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>172</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>174</v>
       </c>
@@ -3625,7 +3625,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>177</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>179</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>181</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>184</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>186</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>188</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>190</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>192</v>
       </c>
@@ -3977,7 +3977,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>195</v>
       </c>
@@ -4021,7 +4021,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>197</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>199</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>201</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>203</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>206</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>208</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>210</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>213</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>215</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>217</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>220</v>
       </c>
@@ -4505,7 +4505,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>223</v>
       </c>
@@ -4549,7 +4549,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>225</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>227</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>229</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>231</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>233</v>
       </c>
@@ -4769,7 +4769,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>235</v>
       </c>
@@ -4813,7 +4813,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>238</v>
       </c>
@@ -4857,7 +4857,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>240</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>243</v>
       </c>
@@ -4945,7 +4945,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>245</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>247</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>249</v>
       </c>
@@ -5077,7 +5077,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>251</v>
       </c>
@@ -5121,7 +5121,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>253</v>
       </c>
@@ -5165,7 +5165,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>255</v>
       </c>
@@ -5209,7 +5209,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>257</v>
       </c>
@@ -5253,7 +5253,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>259</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>261</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>264</v>
       </c>
@@ -5385,7 +5385,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>267</v>
       </c>
@@ -5429,7 +5429,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>270</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>272</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>274</v>
       </c>
@@ -5561,7 +5561,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>277</v>
       </c>
@@ -5605,7 +5605,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>280</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>282</v>
       </c>
@@ -5693,7 +5693,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>284</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>286</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>288</v>
       </c>
@@ -5825,7 +5825,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>291</v>
       </c>
@@ -5869,7 +5869,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>293</v>
       </c>
@@ -5913,7 +5913,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>295</v>
       </c>
@@ -5957,7 +5957,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>297</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>299</v>
       </c>

</xml_diff>